<commit_message>
Conteo de suplementos 18-oct: correcciones de la dueña (JYM 8, multis y magnesio iguales)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MRpmN63Fg2XPVfHVHWCf9v
</commit_message>
<xml_diff>
--- a/docs/operacion/conteos/CONTEO-SUPLEMENTOS-2026-10-18.xlsx
+++ b/docs/operacion/conteos/CONTEO-SUPLEMENTOS-2026-10-18.xlsx
@@ -10,8 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iguales" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="De más en físico" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="De menos en físico" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendiente" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +57,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B45309"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00374151"/>
       </patternFill>
     </fill>
@@ -79,13 +73,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="75" customWidth="1" min="2" max="2"/>
@@ -1249,19 +1242,19 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1128</t>
+          <t>1631</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Hydroxycut Hardcore Elite - MuscleTech - 100 cápsulas</t>
+          <t>Platinum Multi Vitamin - MuscleTech - 180 tabletas</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D38" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -1270,19 +1263,19 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>1125</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Opti-Men - Optimum Nutrition - 150 tabletas / 50 servicios</t>
+          <t>Platinum Multi Vitamin - MuscleTech - 90 tabletas</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
@@ -1291,19 +1284,19 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1128</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Opti-Men - Optimum Nutrition - 90 tabletas / 30 servicios</t>
+          <t>Hydroxycut Hardcore Elite - MuscleTech - 100 cápsulas</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -1312,12 +1305,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1110</t>
+          <t>1003</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Opti-Women - Optimum Nutrition - 120 cápsulas / 60 servicios</t>
+          <t>Opti-Men - Optimum Nutrition - 150 tabletas / 50 servicios</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1333,19 +1326,19 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1109</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Vita Multi-Vitamin - JYM Supplement Science</t>
+          <t>Opti-Men - Optimum Nutrition - 90 tabletas / 30 servicios</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
@@ -1354,19 +1347,19 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1107</t>
+          <t>1110</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Fish Oil - Luma Nutrition - 2,500 mg / 60 softgels</t>
+          <t>Opti-Women - Optimum Nutrition - 120 cápsulas / 60 servicios</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
@@ -1375,19 +1368,19 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1124</t>
+          <t>1694</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Klean Isolate - Klean Athlete - Natural Vanilla / 516 g</t>
+          <t>Magnesium Citrate - NOW - 90 softgels (con glicinato y malato)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
@@ -1396,12 +1389,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1122</t>
+          <t>1109</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Klean Creatine - Klean Athlete - 315 g / polvo</t>
+          <t>Vita Multi-Vitamin - JYM Supplement Science</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1417,19 +1410,19 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1120</t>
+          <t>1107</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Klean Calcium (Citrate) - Klean Athlete - 120 cápsulas</t>
+          <t>Fish Oil - Luma Nutrition - 2,500 mg / 60 softgels</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="D46" t="n">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
@@ -1438,12 +1431,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1117</t>
+          <t>1124</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Klean Zinc - Klean Athlete - Natural Orange / 100 tabletas masticables</t>
+          <t>Klean Isolate - Klean Athlete - Natural Vanilla / 516 g</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1459,19 +1452,19 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1123</t>
+          <t>1122</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Klean Essential Aminos + HMB - Klean Athlete - Orange Cream / 30 servicios</t>
+          <t>Klean Creatine - Klean Athlete - 315 g / polvo</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D48" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
@@ -1480,19 +1473,19 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1116</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Klean Multivitamin - Klean Athlete - 60 tabletas</t>
+          <t>Klean Calcium (Citrate) - Klean Athlete - 120 cápsulas</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
@@ -1501,19 +1494,19 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1118</t>
+          <t>1117</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Klean Magnesium - Klean Athlete - 90 cápsulas vegetarianas</t>
+          <t>Klean Zinc - Klean Athlete - Natural Orange / 100 tabletas masticables</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
@@ -1522,19 +1515,19 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1119</t>
+          <t>1123</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Klean Ashwagandha - Klean Athlete - 60 cápsulas</t>
+          <t>Klean Essential Aminos + HMB - Klean Athlete - Orange Cream / 30 servicios</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
@@ -1543,19 +1536,19 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1115</t>
+          <t>1116</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Klean B-Complex - Klean Athlete - 60 cápsulas vegetarianas</t>
+          <t>Klean Multivitamin - Klean Athlete - 60 tabletas</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D52" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
@@ -1564,12 +1557,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1099</t>
+          <t>1118</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PhedraCut Advanced - USN - 60 cápsulas</t>
+          <t>Klean Magnesium - Klean Athlete - 90 cápsulas vegetarianas</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1579,6 +1572,69 @@
         <v>4</v>
       </c>
       <c r="E53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1119</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Klean Ashwagandha - Klean Athlete - 60 cápsulas</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>6</v>
+      </c>
+      <c r="D54" t="n">
+        <v>6</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1115</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Klean B-Complex - Klean Athlete - 60 cápsulas vegetarianas</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>13</v>
+      </c>
+      <c r="D55" t="n">
+        <v>13</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1099</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PhedraCut Advanced - USN - 60 cápsulas</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1664,7 +1720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="75" customWidth="1" min="2" max="2"/>
@@ -1760,10 +1816,10 @@
         <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="5">
@@ -1847,27 +1903,6 @@
         <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1694</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Magnesium Citrate - NOW - 90 softgels (con glicinato y malato)</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" t="n">
         <v>-2</v>
       </c>
     </row>
@@ -1882,114 +1917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Producto</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Sistema</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Físico</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Diferencia</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Nota</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1631</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Platinum Multi Vitamin - MuscleTech - 180 tabletas</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>La dueña lo chequea en persona</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1125</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Platinum Multi Vitamin - MuscleTech - 90 tabletas</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>La dueña lo chequea en persona</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="75" customWidth="1" min="2" max="2"/>
@@ -2002,42 +1930,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Antes</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Después</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Motivo</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -2171,10 +2099,10 @@
         <v>9</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2326,42 +2254,6 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
-        <is>
-          <t>PENDIENTE de confirmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1694</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Magnesium Citrate - NOW - 90 softgels (con glicinato y malato)</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-2</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Conteo de suplementos (Excel Cloud 18-oct)</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
         <is>
           <t>PENDIENTE de confirmar</t>
         </is>

</xml_diff>

<commit_message>
Conteo de suplementos 18-oct aplicado (8 ajustes) y foto base de la Tienda (122 productos, 577 uds)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MRpmN63Fg2XPVfHVHWCf9v
</commit_message>
<xml_diff>
--- a/docs/operacion/conteos/CONTEO-SUPLEMENTOS-2026-10-18.xlsx
+++ b/docs/operacion/conteos/CONTEO-SUPLEMENTOS-2026-10-18.xlsx
@@ -2003,7 +2003,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>PENDIENTE de confirmar</t>
+          <t>APLICADO 18-oct, verificado 6 veces</t>
         </is>
       </c>
     </row>

</xml_diff>